<commit_message>
Complete RoomifyWeb overhaul: Global Light Mode, UI Bug Fixes, Budget Fixes, Catalog Logic, and E2E Tests
</commit_message>
<xml_diff>
--- a/RoomifyWeb/E2E_Test_Report_RoomifyWeb.xlsx
+++ b/RoomifyWeb/E2E_Test_Report_RoomifyWeb.xlsx
@@ -484,25 +484,25 @@
         <v>104</v>
       </c>
       <c r="C2" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>99.04000000000001</v>
+        <v>100</v>
       </c>
       <c r="F2" t="n">
-        <v>20.83</v>
+        <v>24.7</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:33.437315Z</t>
+          <t>2026-06-15T12:49:44.453349Z</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:54.266140Z</t>
+          <t>2026-06-15T12:50:09.150801Z</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E104"/>
+  <dimension ref="A1:E105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>3.02</v>
+        <v>1.24</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.29</v>
+        <v>0.27</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -600,21 +600,21 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>TC-004</t>
+          <t>TC-003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Catalog</t>
+          <t>Authentication</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Verify Catalog Page Loads</t>
+          <t>Verify Registration Page Renders</t>
         </is>
       </c>
       <c r="D4" t="n">
-        <v>0.16</v>
+        <v>0.18</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -625,21 +625,21 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>TC-005</t>
+          <t>TC-004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Stress Testing</t>
+          <t>Catalog</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #1</t>
+          <t>Verify Catalog Page Loads</t>
         </is>
       </c>
       <c r="D5" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -650,7 +650,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>TC-006</t>
+          <t>TC-005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -660,11 +660,11 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #2</t>
+          <t>Catalog UI Rendering Cycle #1</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>TC-007</t>
+          <t>TC-006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -685,7 +685,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #3</t>
+          <t>Catalog UI Rendering Cycle #2</t>
         </is>
       </c>
       <c r="D7" t="n">
@@ -700,7 +700,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TC-008</t>
+          <t>TC-007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -710,11 +710,11 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #4</t>
+          <t>Catalog UI Rendering Cycle #3</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -725,7 +725,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>TC-009</t>
+          <t>TC-008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -735,11 +735,11 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #5</t>
+          <t>Catalog UI Rendering Cycle #4</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -750,7 +750,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>TC-010</t>
+          <t>TC-009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -760,11 +760,11 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #6</t>
+          <t>Catalog UI Rendering Cycle #5</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -775,7 +775,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TC-011</t>
+          <t>TC-010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -785,7 +785,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #7</t>
+          <t>Catalog UI Rendering Cycle #6</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -800,7 +800,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TC-012</t>
+          <t>TC-011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -810,7 +810,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #8</t>
+          <t>Catalog UI Rendering Cycle #7</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -825,7 +825,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TC-013</t>
+          <t>TC-012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -835,11 +835,11 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #9</t>
+          <t>Catalog UI Rendering Cycle #8</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
@@ -850,7 +850,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TC-014</t>
+          <t>TC-013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -860,7 +860,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #10</t>
+          <t>Catalog UI Rendering Cycle #9</t>
         </is>
       </c>
       <c r="D14" t="n">
@@ -875,7 +875,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TC-015</t>
+          <t>TC-014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -885,7 +885,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #11</t>
+          <t>Catalog UI Rendering Cycle #10</t>
         </is>
       </c>
       <c r="D15" t="n">
@@ -900,7 +900,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>TC-016</t>
+          <t>TC-015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -910,11 +910,11 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #12</t>
+          <t>Catalog UI Rendering Cycle #11</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -925,7 +925,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>TC-017</t>
+          <t>TC-016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -935,11 +935,11 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #13</t>
+          <t>Catalog UI Rendering Cycle #12</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -950,7 +950,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>TC-018</t>
+          <t>TC-017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -960,11 +960,11 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #14</t>
+          <t>Catalog UI Rendering Cycle #13</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>TC-019</t>
+          <t>TC-018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -985,11 +985,11 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #15</t>
+          <t>Catalog UI Rendering Cycle #14</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -1000,7 +1000,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>TC-020</t>
+          <t>TC-019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -1010,11 +1010,11 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #16</t>
+          <t>Catalog UI Rendering Cycle #15</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -1025,7 +1025,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>TC-021</t>
+          <t>TC-020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1035,11 +1035,11 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #17</t>
+          <t>Catalog UI Rendering Cycle #16</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>TC-022</t>
+          <t>TC-021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -1060,11 +1060,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #18</t>
+          <t>Catalog UI Rendering Cycle #17</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -1075,7 +1075,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>TC-023</t>
+          <t>TC-022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1085,11 +1085,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #19</t>
+          <t>Catalog UI Rendering Cycle #18</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -1100,7 +1100,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>TC-024</t>
+          <t>TC-023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1110,7 +1110,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #20</t>
+          <t>Catalog UI Rendering Cycle #19</t>
         </is>
       </c>
       <c r="D24" t="n">
@@ -1125,7 +1125,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>TC-025</t>
+          <t>TC-024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1135,11 +1135,11 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #21</t>
+          <t>Catalog UI Rendering Cycle #20</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.99</v>
+        <v>0.13</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>TC-026</t>
+          <t>TC-025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1160,11 +1160,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #22</t>
+          <t>Catalog UI Rendering Cycle #21</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -1175,7 +1175,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TC-027</t>
+          <t>TC-026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -1185,7 +1185,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #23</t>
+          <t>Catalog UI Rendering Cycle #22</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -1200,7 +1200,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>TC-028</t>
+          <t>TC-027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1210,11 +1210,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #24</t>
+          <t>Catalog UI Rendering Cycle #23</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -1225,7 +1225,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>TC-029</t>
+          <t>TC-028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #25</t>
+          <t>Catalog UI Rendering Cycle #24</t>
         </is>
       </c>
       <c r="D29" t="n">
@@ -1250,7 +1250,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>TC-030</t>
+          <t>TC-029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1260,11 +1260,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #26</t>
+          <t>Catalog UI Rendering Cycle #25</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>TC-031</t>
+          <t>TC-030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -1285,11 +1285,11 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #27</t>
+          <t>Catalog UI Rendering Cycle #26</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -1300,7 +1300,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>TC-032</t>
+          <t>TC-031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -1310,7 +1310,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #28</t>
+          <t>Catalog UI Rendering Cycle #27</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1325,7 +1325,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TC-033</t>
+          <t>TC-032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -1335,11 +1335,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #29</t>
+          <t>Catalog UI Rendering Cycle #28</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>TC-034</t>
+          <t>TC-033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -1360,11 +1360,11 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #30</t>
+          <t>Catalog UI Rendering Cycle #29</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -1375,7 +1375,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>TC-035</t>
+          <t>TC-034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -1385,11 +1385,11 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #31</t>
+          <t>Catalog UI Rendering Cycle #30</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -1400,7 +1400,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>TC-036</t>
+          <t>TC-035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -1410,11 +1410,11 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #32</t>
+          <t>Catalog UI Rendering Cycle #31</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TC-037</t>
+          <t>TC-036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -1435,7 +1435,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #33</t>
+          <t>Catalog UI Rendering Cycle #32</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -1450,7 +1450,7 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>TC-038</t>
+          <t>TC-037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -1460,11 +1460,11 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #34</t>
+          <t>Catalog UI Rendering Cycle #33</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -1475,7 +1475,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>TC-039</t>
+          <t>TC-038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -1485,11 +1485,11 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #35</t>
+          <t>Catalog UI Rendering Cycle #34</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -1500,7 +1500,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TC-040</t>
+          <t>TC-039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -1510,11 +1510,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #36</t>
+          <t>Catalog UI Rendering Cycle #35</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -1525,7 +1525,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>TC-041</t>
+          <t>TC-040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1535,11 +1535,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #37</t>
+          <t>Catalog UI Rendering Cycle #36</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -1550,7 +1550,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>TC-042</t>
+          <t>TC-041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -1560,11 +1560,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #38</t>
+          <t>Catalog UI Rendering Cycle #37</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>TC-043</t>
+          <t>TC-042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1585,11 +1585,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #39</t>
+          <t>Catalog UI Rendering Cycle #38</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -1600,7 +1600,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>TC-044</t>
+          <t>TC-043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -1610,11 +1610,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #40</t>
+          <t>Catalog UI Rendering Cycle #39</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -1625,7 +1625,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>TC-045</t>
+          <t>TC-044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #41</t>
+          <t>Catalog UI Rendering Cycle #40</t>
         </is>
       </c>
       <c r="D45" t="n">
@@ -1650,7 +1650,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>TC-046</t>
+          <t>TC-045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -1660,11 +1660,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #42</t>
+          <t>Catalog UI Rendering Cycle #41</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -1675,7 +1675,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TC-047</t>
+          <t>TC-046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -1685,11 +1685,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #43</t>
+          <t>Catalog UI Rendering Cycle #42</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -1700,7 +1700,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TC-048</t>
+          <t>TC-047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -1710,11 +1710,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #44</t>
+          <t>Catalog UI Rendering Cycle #43</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>TC-049</t>
+          <t>TC-048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -1735,11 +1735,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #45</t>
+          <t>Catalog UI Rendering Cycle #44</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -1750,7 +1750,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>TC-050</t>
+          <t>TC-049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -1760,11 +1760,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #46</t>
+          <t>Catalog UI Rendering Cycle #45</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.16</v>
+        <v>0.22</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -1775,7 +1775,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TC-051</t>
+          <t>TC-050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -1785,11 +1785,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #47</t>
+          <t>Catalog UI Rendering Cycle #46</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -1800,7 +1800,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>TC-052</t>
+          <t>TC-051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -1810,11 +1810,11 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #48</t>
+          <t>Catalog UI Rendering Cycle #47</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -1825,7 +1825,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>TC-053</t>
+          <t>TC-052</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -1835,11 +1835,11 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #49</t>
+          <t>Catalog UI Rendering Cycle #48</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -1850,7 +1850,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>TC-054</t>
+          <t>TC-053</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -1860,11 +1860,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #50</t>
+          <t>Catalog UI Rendering Cycle #49</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1875,7 +1875,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>TC-055</t>
+          <t>TC-054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -1885,11 +1885,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #51</t>
+          <t>Catalog UI Rendering Cycle #50</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.12</v>
+        <v>0.28</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -1900,7 +1900,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TC-056</t>
+          <t>TC-055</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -1910,11 +1910,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #52</t>
+          <t>Catalog UI Rendering Cycle #51</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.14</v>
+        <v>0.24</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -1925,7 +1925,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>TC-057</t>
+          <t>TC-056</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -1935,11 +1935,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #53</t>
+          <t>Catalog UI Rendering Cycle #52</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.12</v>
+        <v>0.19</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -1950,7 +1950,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TC-058</t>
+          <t>TC-057</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -1960,11 +1960,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #54</t>
+          <t>Catalog UI Rendering Cycle #53</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -1975,7 +1975,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>TC-059</t>
+          <t>TC-058</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -1985,11 +1985,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #55</t>
+          <t>Catalog UI Rendering Cycle #54</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2000,7 +2000,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TC-060</t>
+          <t>TC-059</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -2010,11 +2010,11 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #56</t>
+          <t>Catalog UI Rendering Cycle #55</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -2025,7 +2025,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TC-061</t>
+          <t>TC-060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -2035,11 +2035,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #57</t>
+          <t>Catalog UI Rendering Cycle #56</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -2050,7 +2050,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>TC-062</t>
+          <t>TC-061</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -2060,11 +2060,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #58</t>
+          <t>Catalog UI Rendering Cycle #57</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -2075,7 +2075,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>TC-063</t>
+          <t>TC-062</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -2085,11 +2085,11 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #59</t>
+          <t>Catalog UI Rendering Cycle #58</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -2100,7 +2100,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>TC-064</t>
+          <t>TC-063</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -2110,11 +2110,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #60</t>
+          <t>Catalog UI Rendering Cycle #59</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -2125,7 +2125,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>TC-065</t>
+          <t>TC-064</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -2135,11 +2135,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #61</t>
+          <t>Catalog UI Rendering Cycle #60</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.14</v>
+        <v>0.15</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -2150,7 +2150,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>TC-066</t>
+          <t>TC-065</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #62</t>
+          <t>Catalog UI Rendering Cycle #61</t>
         </is>
       </c>
       <c r="D66" t="n">
@@ -2175,7 +2175,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>TC-067</t>
+          <t>TC-066</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -2185,11 +2185,11 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #63</t>
+          <t>Catalog UI Rendering Cycle #62</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -2200,7 +2200,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>TC-068</t>
+          <t>TC-067</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #64</t>
+          <t>Catalog UI Rendering Cycle #63</t>
         </is>
       </c>
       <c r="D68" t="n">
@@ -2225,7 +2225,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TC-069</t>
+          <t>TC-068</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -2235,7 +2235,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #65</t>
+          <t>Catalog UI Rendering Cycle #64</t>
         </is>
       </c>
       <c r="D69" t="n">
@@ -2250,7 +2250,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TC-070</t>
+          <t>TC-069</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -2260,11 +2260,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #66</t>
+          <t>Catalog UI Rendering Cycle #65</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -2275,7 +2275,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>TC-071</t>
+          <t>TC-070</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -2285,11 +2285,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #67</t>
+          <t>Catalog UI Rendering Cycle #66</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -2300,7 +2300,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>TC-072</t>
+          <t>TC-071</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -2310,11 +2310,11 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #68</t>
+          <t>Catalog UI Rendering Cycle #67</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -2325,7 +2325,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>TC-073</t>
+          <t>TC-072</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -2335,11 +2335,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #69</t>
+          <t>Catalog UI Rendering Cycle #68</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -2350,7 +2350,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>TC-074</t>
+          <t>TC-073</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -2360,11 +2360,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #70</t>
+          <t>Catalog UI Rendering Cycle #69</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -2375,7 +2375,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>TC-075</t>
+          <t>TC-074</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -2385,11 +2385,11 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #71</t>
+          <t>Catalog UI Rendering Cycle #70</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -2400,7 +2400,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>TC-076</t>
+          <t>TC-075</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -2410,7 +2410,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #72</t>
+          <t>Catalog UI Rendering Cycle #71</t>
         </is>
       </c>
       <c r="D76" t="n">
@@ -2425,7 +2425,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>TC-077</t>
+          <t>TC-076</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -2435,11 +2435,11 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #73</t>
+          <t>Catalog UI Rendering Cycle #72</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -2450,7 +2450,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>TC-078</t>
+          <t>TC-077</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -2460,11 +2460,11 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #74</t>
+          <t>Catalog UI Rendering Cycle #73</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -2475,7 +2475,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>TC-079</t>
+          <t>TC-078</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -2485,11 +2485,11 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #75</t>
+          <t>Catalog UI Rendering Cycle #74</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -2500,7 +2500,7 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>TC-080</t>
+          <t>TC-079</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -2510,11 +2510,11 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #76</t>
+          <t>Catalog UI Rendering Cycle #75</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>0.12</v>
+        <v>0.14</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -2525,7 +2525,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>TC-081</t>
+          <t>TC-080</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -2535,7 +2535,7 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #77</t>
+          <t>Catalog UI Rendering Cycle #76</t>
         </is>
       </c>
       <c r="D81" t="n">
@@ -2550,7 +2550,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>TC-082</t>
+          <t>TC-081</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -2560,11 +2560,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #78</t>
+          <t>Catalog UI Rendering Cycle #77</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -2575,7 +2575,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>TC-083</t>
+          <t>TC-082</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -2585,11 +2585,11 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #79</t>
+          <t>Catalog UI Rendering Cycle #78</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -2600,7 +2600,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>TC-084</t>
+          <t>TC-083</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -2610,7 +2610,7 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #80</t>
+          <t>Catalog UI Rendering Cycle #79</t>
         </is>
       </c>
       <c r="D84" t="n">
@@ -2625,7 +2625,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>TC-085</t>
+          <t>TC-084</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -2635,11 +2635,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #81</t>
+          <t>Catalog UI Rendering Cycle #80</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -2650,7 +2650,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>TC-086</t>
+          <t>TC-085</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -2660,11 +2660,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #82</t>
+          <t>Catalog UI Rendering Cycle #81</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -2675,7 +2675,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>TC-087</t>
+          <t>TC-086</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -2685,11 +2685,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #83</t>
+          <t>Catalog UI Rendering Cycle #82</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -2700,7 +2700,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>TC-088</t>
+          <t>TC-087</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -2710,11 +2710,11 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #84</t>
+          <t>Catalog UI Rendering Cycle #83</t>
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -2725,7 +2725,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>TC-089</t>
+          <t>TC-088</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -2735,11 +2735,11 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #85</t>
+          <t>Catalog UI Rendering Cycle #84</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -2750,7 +2750,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>TC-090</t>
+          <t>TC-089</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -2760,11 +2760,11 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #86</t>
+          <t>Catalog UI Rendering Cycle #85</t>
         </is>
       </c>
       <c r="D90" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -2775,7 +2775,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>TC-091</t>
+          <t>TC-090</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -2785,11 +2785,11 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #87</t>
+          <t>Catalog UI Rendering Cycle #86</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0.12</v>
+        <v>0.16</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -2800,7 +2800,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>TC-092</t>
+          <t>TC-091</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -2810,11 +2810,11 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #88</t>
+          <t>Catalog UI Rendering Cycle #87</t>
         </is>
       </c>
       <c r="D92" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -2825,7 +2825,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>TC-093</t>
+          <t>TC-092</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -2835,11 +2835,11 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #89</t>
+          <t>Catalog UI Rendering Cycle #88</t>
         </is>
       </c>
       <c r="D93" t="n">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -2850,7 +2850,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>TC-094</t>
+          <t>TC-093</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -2860,11 +2860,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #90</t>
+          <t>Catalog UI Rendering Cycle #89</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -2875,7 +2875,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TC-095</t>
+          <t>TC-094</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -2885,11 +2885,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #91</t>
+          <t>Catalog UI Rendering Cycle #90</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.12</v>
+        <v>0.15</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -2900,7 +2900,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>TC-096</t>
+          <t>TC-095</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -2910,11 +2910,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #92</t>
+          <t>Catalog UI Rendering Cycle #91</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0.13</v>
+        <v>0.18</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -2925,7 +2925,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>TC-097</t>
+          <t>TC-096</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -2935,11 +2935,11 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #93</t>
+          <t>Catalog UI Rendering Cycle #92</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -2950,7 +2950,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>TC-098</t>
+          <t>TC-097</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -2960,11 +2960,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #94</t>
+          <t>Catalog UI Rendering Cycle #93</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -2975,7 +2975,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>TC-099</t>
+          <t>TC-098</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -2985,11 +2985,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #95</t>
+          <t>Catalog UI Rendering Cycle #94</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -3000,7 +3000,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>TC-100</t>
+          <t>TC-099</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #96</t>
+          <t>Catalog UI Rendering Cycle #95</t>
         </is>
       </c>
       <c r="D100" t="n">
@@ -3025,7 +3025,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>TC-101</t>
+          <t>TC-100</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -3035,11 +3035,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #97</t>
+          <t>Catalog UI Rendering Cycle #96</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -3050,7 +3050,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>TC-102</t>
+          <t>TC-101</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -3060,11 +3060,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #98</t>
+          <t>Catalog UI Rendering Cycle #97</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.13</v>
+        <v>0.15</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -3075,7 +3075,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>TC-103</t>
+          <t>TC-102</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -3085,11 +3085,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Catalog UI Rendering Cycle #99</t>
+          <t>Catalog UI Rendering Cycle #98</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -3100,23 +3100,48 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
+          <t>TC-103</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Stress Testing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Catalog UI Rendering Cycle #99</t>
+        </is>
+      </c>
+      <c r="D104" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
           <t>TC-104</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
-        <is>
-          <t>Stress Testing</t>
-        </is>
-      </c>
-      <c r="C104" t="inlineStr">
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Stress Testing</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
         <is>
           <t>Catalog UI Rendering Cycle #100</t>
         </is>
       </c>
-      <c r="D104" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="E104" t="inlineStr">
+      <c r="D105" t="n">
+        <v>0.9399999999999999</v>
+      </c>
+      <c r="E105" t="inlineStr">
         <is>
           <t>Passed</t>
         </is>
@@ -3133,70 +3158,9 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:A1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Test Name</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Error</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Timestamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TC-003</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Authentication</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Verify Registration Page Renders</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Failed</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>2026-06-15T04:48:54.266140Z</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3230,7 +3194,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:33.437396Z</t>
+          <t>2026-06-15T12:49:44.453445Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -3247,7 +3211,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:36.458256Z</t>
+          <t>2026-06-15T12:49:45.697335Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -3257,14 +3221,14 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Test TC-001 Passed in 3.02s</t>
+          <t>Test TC-001 Passed in 1.24s</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:36.458335Z</t>
+          <t>2026-06-15T12:49:45.697402Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -3281,7 +3245,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:36.748328Z</t>
+          <t>2026-06-15T12:49:45.971628Z</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -3291,14 +3255,14 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Test TC-002 Passed in 0.29s</t>
+          <t>Test TC-002 Passed in 0.27s</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:36.748401Z</t>
+          <t>2026-06-15T12:49:45.971697Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -3315,24 +3279,24 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:36.990304Z</t>
+          <t>2026-06-15T12:49:46.155372Z</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>ERROR</t>
+          <t>SUCCESS</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Test TC-003 Failed: </t>
+          <t>Test TC-003 Passed in 0.18s</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:36.990362Z</t>
+          <t>2026-06-15T12:49:46.155423Z</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -3349,7 +3313,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.151195Z</t>
+          <t>2026-06-15T12:49:46.310543Z</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -3366,7 +3330,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.151254Z</t>
+          <t>2026-06-15T12:49:46.310602Z</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -3383,7 +3347,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.299509Z</t>
+          <t>2026-06-15T12:49:46.466780Z</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -3393,14 +3357,14 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Test TC-005 Passed in 0.15s</t>
+          <t>Test TC-005 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.299570Z</t>
+          <t>2026-06-15T12:49:46.466848Z</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -3417,7 +3381,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.432475Z</t>
+          <t>2026-06-15T12:49:46.598060Z</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -3434,7 +3398,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.432538Z</t>
+          <t>2026-06-15T12:49:46.598115Z</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -3451,7 +3415,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.560496Z</t>
+          <t>2026-06-15T12:49:46.725215Z</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3468,7 +3432,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.560552Z</t>
+          <t>2026-06-15T12:49:46.725272Z</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -3485,7 +3449,7 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.704696Z</t>
+          <t>2026-06-15T12:49:46.860699Z</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -3502,7 +3466,7 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.704754Z</t>
+          <t>2026-06-15T12:49:46.860781Z</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3519,7 +3483,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.838000Z</t>
+          <t>2026-06-15T12:49:47.002656Z</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3529,14 +3493,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Test TC-009 Passed in 0.13s</t>
+          <t>Test TC-009 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.838063Z</t>
+          <t>2026-06-15T12:49:47.002711Z</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3553,7 +3517,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.984265Z</t>
+          <t>2026-06-15T12:49:47.144614Z</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3563,14 +3527,14 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Test TC-010 Passed in 0.15s</t>
+          <t>Test TC-010 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:37.984321Z</t>
+          <t>2026-06-15T12:49:47.144680Z</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3587,7 +3551,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.119365Z</t>
+          <t>2026-06-15T12:49:47.278110Z</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3597,14 +3561,14 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Test TC-011 Passed in 0.14s</t>
+          <t>Test TC-011 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.119490Z</t>
+          <t>2026-06-15T12:49:47.278166Z</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -3621,7 +3585,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.247349Z</t>
+          <t>2026-06-15T12:49:47.407172Z</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -3638,7 +3602,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.247405Z</t>
+          <t>2026-06-15T12:49:47.407239Z</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -3655,7 +3619,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.407536Z</t>
+          <t>2026-06-15T12:49:47.539556Z</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -3665,14 +3629,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Test TC-013 Passed in 0.16s</t>
+          <t>Test TC-013 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.407596Z</t>
+          <t>2026-06-15T12:49:47.539612Z</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3689,7 +3653,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.538885Z</t>
+          <t>2026-06-15T12:49:47.668552Z</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3706,7 +3670,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.538945Z</t>
+          <t>2026-06-15T12:49:47.668607Z</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -3723,7 +3687,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.669651Z</t>
+          <t>2026-06-15T12:49:47.801799Z</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -3740,7 +3704,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.669709Z</t>
+          <t>2026-06-15T12:49:47.801871Z</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -3757,7 +3721,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.811973Z</t>
+          <t>2026-06-15T12:49:47.940091Z</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -3774,7 +3738,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.812030Z</t>
+          <t>2026-06-15T12:49:47.940147Z</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -3791,7 +3755,7 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.941222Z</t>
+          <t>2026-06-15T12:49:48.066038Z</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
@@ -3808,7 +3772,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:38.941283Z</t>
+          <t>2026-06-15T12:49:48.066107Z</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
@@ -3825,7 +3789,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.087011Z</t>
+          <t>2026-06-15T12:49:48.194001Z</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -3835,14 +3799,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Test TC-018 Passed in 0.15s</t>
+          <t>Test TC-018 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.087066Z</t>
+          <t>2026-06-15T12:49:48.194057Z</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
@@ -3859,7 +3823,7 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.243578Z</t>
+          <t>2026-06-15T12:49:48.323227Z</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
@@ -3869,14 +3833,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Test TC-019 Passed in 0.16s</t>
+          <t>Test TC-019 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.243658Z</t>
+          <t>2026-06-15T12:49:48.323284Z</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -3893,7 +3857,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.391358Z</t>
+          <t>2026-06-15T12:49:48.474801Z</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -3910,7 +3874,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.391417Z</t>
+          <t>2026-06-15T12:49:48.474873Z</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -3927,7 +3891,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.512033Z</t>
+          <t>2026-06-15T12:49:48.617665Z</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -3937,14 +3901,14 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Test TC-021 Passed in 0.12s</t>
+          <t>Test TC-021 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.512089Z</t>
+          <t>2026-06-15T12:49:48.617729Z</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -3961,7 +3925,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.635886Z</t>
+          <t>2026-06-15T12:49:48.754427Z</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -3971,14 +3935,14 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Test TC-022 Passed in 0.12s</t>
+          <t>Test TC-022 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.635943Z</t>
+          <t>2026-06-15T12:49:48.754484Z</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -3995,7 +3959,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.761666Z</t>
+          <t>2026-06-15T12:49:48.884952Z</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -4012,7 +3976,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.761724Z</t>
+          <t>2026-06-15T12:49:48.885036Z</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -4029,7 +3993,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.886874Z</t>
+          <t>2026-06-15T12:49:49.016618Z</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -4046,7 +4010,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:39.886952Z</t>
+          <t>2026-06-15T12:49:49.016686Z</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -4063,7 +4027,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:40.877788Z</t>
+          <t>2026-06-15T12:49:49.158624Z</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -4073,14 +4037,14 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Test TC-025 Passed in 0.99s</t>
+          <t>Test TC-025 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:40.877843Z</t>
+          <t>2026-06-15T12:49:49.158679Z</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -4097,7 +4061,7 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.011006Z</t>
+          <t>2026-06-15T12:49:49.286952Z</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
@@ -4114,7 +4078,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.011061Z</t>
+          <t>2026-06-15T12:49:49.287011Z</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -4131,7 +4095,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.143449Z</t>
+          <t>2026-06-15T12:49:49.432908Z</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -4141,14 +4105,14 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Test TC-027 Passed in 0.13s</t>
+          <t>Test TC-027 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.143507Z</t>
+          <t>2026-06-15T12:49:49.432965Z</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -4165,7 +4129,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.279125Z</t>
+          <t>2026-06-15T12:49:49.570944Z</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -4182,7 +4146,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.279179Z</t>
+          <t>2026-06-15T12:49:49.571014Z</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -4199,7 +4163,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.419419Z</t>
+          <t>2026-06-15T12:49:49.725263Z</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4209,14 +4173,14 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Test TC-029 Passed in 0.14s</t>
+          <t>Test TC-029 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.419475Z</t>
+          <t>2026-06-15T12:49:49.725328Z</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4233,7 +4197,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.538799Z</t>
+          <t>2026-06-15T12:49:49.859136Z</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -4243,14 +4207,14 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Test TC-030 Passed in 0.12s</t>
+          <t>Test TC-030 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.538859Z</t>
+          <t>2026-06-15T12:49:49.859221Z</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4267,7 +4231,7 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.661712Z</t>
+          <t>2026-06-15T12:49:49.988448Z</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
@@ -4277,14 +4241,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Test TC-031 Passed in 0.12s</t>
+          <t>Test TC-031 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.661767Z</t>
+          <t>2026-06-15T12:49:49.988508Z</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -4301,7 +4265,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.790941Z</t>
+          <t>2026-06-15T12:49:50.117221Z</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -4318,7 +4282,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.791041Z</t>
+          <t>2026-06-15T12:49:50.117299Z</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
@@ -4335,7 +4299,7 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.926473Z</t>
+          <t>2026-06-15T12:49:50.245696Z</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
@@ -4345,14 +4309,14 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Test TC-033 Passed in 0.14s</t>
+          <t>Test TC-033 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:41.926538Z</t>
+          <t>2026-06-15T12:49:50.245750Z</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -4369,7 +4333,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.070745Z</t>
+          <t>2026-06-15T12:49:50.386258Z</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -4386,7 +4350,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.070825Z</t>
+          <t>2026-06-15T12:49:50.386314Z</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -4403,7 +4367,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.216252Z</t>
+          <t>2026-06-15T12:49:50.517858Z</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -4413,14 +4377,14 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Test TC-035 Passed in 0.15s</t>
+          <t>Test TC-035 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.216311Z</t>
+          <t>2026-06-15T12:49:50.517912Z</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -4437,7 +4401,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.337288Z</t>
+          <t>2026-06-15T12:49:50.643290Z</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -4447,14 +4411,14 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Test TC-036 Passed in 0.12s</t>
+          <t>Test TC-036 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.337347Z</t>
+          <t>2026-06-15T12:49:50.643347Z</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -4471,7 +4435,7 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.463240Z</t>
+          <t>2026-06-15T12:49:50.773385Z</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
@@ -4488,7 +4452,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.463330Z</t>
+          <t>2026-06-15T12:49:50.773443Z</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -4505,7 +4469,7 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.600139Z</t>
+          <t>2026-06-15T12:49:50.913650Z</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
@@ -4522,7 +4486,7 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.600195Z</t>
+          <t>2026-06-15T12:49:50.913706Z</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
@@ -4539,7 +4503,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.720595Z</t>
+          <t>2026-06-15T12:49:51.043688Z</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -4549,14 +4513,14 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Test TC-039 Passed in 0.12s</t>
+          <t>Test TC-039 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.720654Z</t>
+          <t>2026-06-15T12:49:51.043745Z</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
@@ -4573,7 +4537,7 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.842428Z</t>
+          <t>2026-06-15T12:49:51.187827Z</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
@@ -4583,14 +4547,14 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Test TC-040 Passed in 0.12s</t>
+          <t>Test TC-040 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.842485Z</t>
+          <t>2026-06-15T12:49:51.187894Z</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -4607,7 +4571,7 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.959937Z</t>
+          <t>2026-06-15T12:49:51.343550Z</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
@@ -4617,14 +4581,14 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Test TC-041 Passed in 0.12s</t>
+          <t>Test TC-041 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:42.959994Z</t>
+          <t>2026-06-15T12:49:51.343606Z</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -4641,7 +4605,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.083804Z</t>
+          <t>2026-06-15T12:49:51.506735Z</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -4651,14 +4615,14 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Test TC-042 Passed in 0.12s</t>
+          <t>Test TC-042 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.083862Z</t>
+          <t>2026-06-15T12:49:51.506820Z</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -4675,7 +4639,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.229159Z</t>
+          <t>2026-06-15T12:49:51.672868Z</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -4685,14 +4649,14 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Test TC-043 Passed in 0.15s</t>
+          <t>Test TC-043 Passed in 0.17s</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.229231Z</t>
+          <t>2026-06-15T12:49:51.672937Z</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
@@ -4709,7 +4673,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.362280Z</t>
+          <t>2026-06-15T12:49:51.806784Z</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
@@ -4726,7 +4690,7 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.362335Z</t>
+          <t>2026-06-15T12:49:51.806849Z</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
@@ -4743,7 +4707,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.494227Z</t>
+          <t>2026-06-15T12:49:51.970906Z</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
@@ -4753,14 +4717,14 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Test TC-045 Passed in 0.13s</t>
+          <t>Test TC-045 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.494290Z</t>
+          <t>2026-06-15T12:49:51.971012Z</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -4777,7 +4741,7 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.613190Z</t>
+          <t>2026-06-15T12:49:52.106766Z</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
@@ -4787,14 +4751,14 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Test TC-046 Passed in 0.12s</t>
+          <t>Test TC-046 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.613247Z</t>
+          <t>2026-06-15T12:49:52.106832Z</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -4811,7 +4775,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.746507Z</t>
+          <t>2026-06-15T12:49:52.260623Z</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -4821,14 +4785,14 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Test TC-047 Passed in 0.13s</t>
+          <t>Test TC-047 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.746563Z</t>
+          <t>2026-06-15T12:49:52.260678Z</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -4845,7 +4809,7 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.873174Z</t>
+          <t>2026-06-15T12:49:52.418126Z</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
@@ -4855,14 +4819,14 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Test TC-048 Passed in 0.13s</t>
+          <t>Test TC-048 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:43.873237Z</t>
+          <t>2026-06-15T12:49:52.418393Z</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -4879,7 +4843,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.006155Z</t>
+          <t>2026-06-15T12:49:52.633651Z</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -4889,14 +4853,14 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Test TC-049 Passed in 0.13s</t>
+          <t>Test TC-049 Passed in 0.22s</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.006237Z</t>
+          <t>2026-06-15T12:49:52.633722Z</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -4913,7 +4877,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.162382Z</t>
+          <t>2026-06-15T12:49:52.774284Z</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -4923,14 +4887,14 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Test TC-050 Passed in 0.16s</t>
+          <t>Test TC-050 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.162466Z</t>
+          <t>2026-06-15T12:49:52.774348Z</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -4947,7 +4911,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.314927Z</t>
+          <t>2026-06-15T12:49:52.928860Z</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -4964,7 +4928,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.315015Z</t>
+          <t>2026-06-15T12:49:52.928931Z</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -4981,7 +4945,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.478542Z</t>
+          <t>2026-06-15T12:49:53.110418Z</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -4991,14 +4955,14 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Test TC-052 Passed in 0.16s</t>
+          <t>Test TC-052 Passed in 0.18s</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.478597Z</t>
+          <t>2026-06-15T12:49:53.110488Z</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -5015,7 +4979,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.622874Z</t>
+          <t>2026-06-15T12:49:53.302426Z</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -5025,14 +4989,14 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Test TC-053 Passed in 0.14s</t>
+          <t>Test TC-053 Passed in 0.19s</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.622937Z</t>
+          <t>2026-06-15T12:49:53.302498Z</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -5049,7 +5013,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.775366Z</t>
+          <t>2026-06-15T12:49:53.580126Z</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -5059,14 +5023,14 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Test TC-054 Passed in 0.15s</t>
+          <t>Test TC-054 Passed in 0.28s</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.775422Z</t>
+          <t>2026-06-15T12:49:53.580209Z</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -5083,7 +5047,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.899340Z</t>
+          <t>2026-06-15T12:49:53.817317Z</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -5093,14 +5057,14 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Test TC-055 Passed in 0.12s</t>
+          <t>Test TC-055 Passed in 0.24s</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:44.899401Z</t>
+          <t>2026-06-15T12:49:53.817384Z</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -5117,7 +5081,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.036374Z</t>
+          <t>2026-06-15T12:49:54.007166Z</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -5127,14 +5091,14 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Test TC-056 Passed in 0.14s</t>
+          <t>Test TC-056 Passed in 0.19s</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.036431Z</t>
+          <t>2026-06-15T12:49:54.007235Z</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -5151,7 +5115,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.158817Z</t>
+          <t>2026-06-15T12:49:54.204883Z</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -5161,14 +5125,14 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Test TC-057 Passed in 0.12s</t>
+          <t>Test TC-057 Passed in 0.2s</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.158873Z</t>
+          <t>2026-06-15T12:49:54.204945Z</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -5185,7 +5149,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.287085Z</t>
+          <t>2026-06-15T12:49:54.431565Z</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -5195,14 +5159,14 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Test TC-058 Passed in 0.13s</t>
+          <t>Test TC-058 Passed in 0.23s</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.287143Z</t>
+          <t>2026-06-15T12:49:54.431636Z</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -5219,7 +5183,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.412993Z</t>
+          <t>2026-06-15T12:49:54.581809Z</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -5229,14 +5193,14 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>Test TC-059 Passed in 0.13s</t>
+          <t>Test TC-059 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.413102Z</t>
+          <t>2026-06-15T12:49:54.581893Z</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
@@ -5253,7 +5217,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.539890Z</t>
+          <t>2026-06-15T12:49:54.716425Z</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
@@ -5270,7 +5234,7 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.539959Z</t>
+          <t>2026-06-15T12:49:54.716509Z</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
@@ -5287,7 +5251,7 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.681538Z</t>
+          <t>2026-06-15T12:49:54.874708Z</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
@@ -5297,14 +5261,14 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>Test TC-061 Passed in 0.14s</t>
+          <t>Test TC-061 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.681621Z</t>
+          <t>2026-06-15T12:49:54.874801Z</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -5321,7 +5285,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.805629Z</t>
+          <t>2026-06-15T12:49:55.031506Z</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -5331,14 +5295,14 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>Test TC-062 Passed in 0.12s</t>
+          <t>Test TC-062 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.805685Z</t>
+          <t>2026-06-15T12:49:55.031577Z</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -5355,7 +5319,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.925532Z</t>
+          <t>2026-06-15T12:49:55.180551Z</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -5365,14 +5329,14 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>Test TC-063 Passed in 0.12s</t>
+          <t>Test TC-063 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:45.925588Z</t>
+          <t>2026-06-15T12:49:55.180634Z</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -5389,7 +5353,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.046515Z</t>
+          <t>2026-06-15T12:49:55.331467Z</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -5399,14 +5363,14 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>Test TC-064 Passed in 0.12s</t>
+          <t>Test TC-064 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.046571Z</t>
+          <t>2026-06-15T12:49:55.331549Z</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -5423,7 +5387,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.183504Z</t>
+          <t>2026-06-15T12:49:55.493518Z</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -5433,14 +5397,14 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Test TC-065 Passed in 0.14s</t>
+          <t>Test TC-065 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.183563Z</t>
+          <t>2026-06-15T12:49:55.493583Z</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
@@ -5457,7 +5421,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.342652Z</t>
+          <t>2026-06-15T12:49:55.624311Z</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -5467,14 +5431,14 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>Test TC-066 Passed in 0.16s</t>
+          <t>Test TC-066 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.342789Z</t>
+          <t>2026-06-15T12:49:55.624367Z</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
@@ -5491,7 +5455,7 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.514320Z</t>
+          <t>2026-06-15T12:49:55.750971Z</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
@@ -5501,14 +5465,14 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>Test TC-067 Passed in 0.17s</t>
+          <t>Test TC-067 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.514394Z</t>
+          <t>2026-06-15T12:49:55.751047Z</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
@@ -5525,7 +5489,7 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.643380Z</t>
+          <t>2026-06-15T12:49:55.878746Z</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -5542,7 +5506,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.643436Z</t>
+          <t>2026-06-15T12:49:55.878826Z</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -5559,7 +5523,7 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.774694Z</t>
+          <t>2026-06-15T12:49:56.008111Z</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
@@ -5576,7 +5540,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.774769Z</t>
+          <t>2026-06-15T12:49:56.008169Z</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -5593,7 +5557,7 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.919520Z</t>
+          <t>2026-06-15T12:49:56.154590Z</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
@@ -5603,14 +5567,14 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>Test TC-070 Passed in 0.14s</t>
+          <t>Test TC-070 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:46.919575Z</t>
+          <t>2026-06-15T12:49:56.154646Z</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
@@ -5627,7 +5591,7 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.045968Z</t>
+          <t>2026-06-15T12:49:56.288534Z</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
@@ -5644,7 +5608,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.046072Z</t>
+          <t>2026-06-15T12:49:56.288614Z</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
@@ -5661,7 +5625,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.169763Z</t>
+          <t>2026-06-15T12:49:56.427160Z</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -5671,14 +5635,14 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Test TC-072 Passed in 0.12s</t>
+          <t>Test TC-072 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.169818Z</t>
+          <t>2026-06-15T12:49:56.427217Z</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
@@ -5695,7 +5659,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.299352Z</t>
+          <t>2026-06-15T12:49:56.551864Z</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
@@ -5705,14 +5669,14 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Test TC-073 Passed in 0.13s</t>
+          <t>Test TC-073 Passed in 0.12s</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.299416Z</t>
+          <t>2026-06-15T12:49:56.551919Z</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
@@ -5729,7 +5693,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.447732Z</t>
+          <t>2026-06-15T12:49:56.690982Z</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
@@ -5739,14 +5703,14 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Test TC-074 Passed in 0.15s</t>
+          <t>Test TC-074 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.447794Z</t>
+          <t>2026-06-15T12:49:56.691051Z</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -5763,7 +5727,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.573130Z</t>
+          <t>2026-06-15T12:49:56.821909Z</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -5780,7 +5744,7 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.573254Z</t>
+          <t>2026-06-15T12:49:56.821970Z</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
@@ -5797,7 +5761,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.698604Z</t>
+          <t>2026-06-15T12:49:56.949334Z</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
@@ -5814,7 +5778,7 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.698668Z</t>
+          <t>2026-06-15T12:49:56.949388Z</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
@@ -5831,7 +5795,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.820064Z</t>
+          <t>2026-06-15T12:49:57.088205Z</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
@@ -5841,14 +5805,14 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Test TC-077 Passed in 0.12s</t>
+          <t>Test TC-077 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.820127Z</t>
+          <t>2026-06-15T12:49:57.088285Z</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
@@ -5865,7 +5829,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.946573Z</t>
+          <t>2026-06-15T12:49:57.215728Z</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -5882,7 +5846,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:47.946633Z</t>
+          <t>2026-06-15T12:49:57.215798Z</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -5899,7 +5863,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.084401Z</t>
+          <t>2026-06-15T12:49:57.357643Z</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
@@ -5916,7 +5880,7 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.084457Z</t>
+          <t>2026-06-15T12:49:57.357714Z</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
@@ -5933,7 +5897,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.208478Z</t>
+          <t>2026-06-15T12:49:57.488532Z</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -5943,14 +5907,14 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Test TC-080 Passed in 0.12s</t>
+          <t>Test TC-080 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.208538Z</t>
+          <t>2026-06-15T12:49:57.488588Z</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
@@ -5967,7 +5931,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.342718Z</t>
+          <t>2026-06-15T12:49:57.616891Z</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
@@ -5984,7 +5948,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.342907Z</t>
+          <t>2026-06-15T12:49:57.617042Z</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -6001,7 +5965,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.486893Z</t>
+          <t>2026-06-15T12:49:57.747540Z</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
@@ -6011,14 +5975,14 @@
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Test TC-082 Passed in 0.14s</t>
+          <t>Test TC-082 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.487016Z</t>
+          <t>2026-06-15T12:49:57.747595Z</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
@@ -6035,7 +5999,7 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.646672Z</t>
+          <t>2026-06-15T12:49:57.888260Z</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
@@ -6045,14 +6009,14 @@
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Test TC-083 Passed in 0.16s</t>
+          <t>Test TC-083 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.646727Z</t>
+          <t>2026-06-15T12:49:57.888330Z</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -6069,7 +6033,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.781943Z</t>
+          <t>2026-06-15T12:49:58.023636Z</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -6086,7 +6050,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.782020Z</t>
+          <t>2026-06-15T12:49:58.023693Z</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -6103,7 +6067,7 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.929523Z</t>
+          <t>2026-06-15T12:49:58.154440Z</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
@@ -6113,14 +6077,14 @@
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Test TC-085 Passed in 0.15s</t>
+          <t>Test TC-085 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:48.929580Z</t>
+          <t>2026-06-15T12:49:58.154498Z</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -6137,7 +6101,7 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.079687Z</t>
+          <t>2026-06-15T12:49:58.288986Z</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
@@ -6147,14 +6111,14 @@
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Test TC-086 Passed in 0.15s</t>
+          <t>Test TC-086 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.079747Z</t>
+          <t>2026-06-15T12:49:58.289061Z</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
@@ -6171,7 +6135,7 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.232939Z</t>
+          <t>2026-06-15T12:49:58.422598Z</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
@@ -6181,14 +6145,14 @@
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Test TC-087 Passed in 0.15s</t>
+          <t>Test TC-087 Passed in 0.13s</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.233015Z</t>
+          <t>2026-06-15T12:49:58.422655Z</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
@@ -6205,7 +6169,7 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.430822Z</t>
+          <t>2026-06-15T12:49:58.570939Z</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
@@ -6215,14 +6179,14 @@
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Test TC-088 Passed in 0.2s</t>
+          <t>Test TC-088 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.431145Z</t>
+          <t>2026-06-15T12:49:58.571003Z</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
@@ -6239,7 +6203,7 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.622311Z</t>
+          <t>2026-06-15T12:49:58.727636Z</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
@@ -6249,14 +6213,14 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Test TC-089 Passed in 0.19s</t>
+          <t>Test TC-089 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.622366Z</t>
+          <t>2026-06-15T12:49:58.727703Z</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
@@ -6273,7 +6237,7 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.759330Z</t>
+          <t>2026-06-15T12:49:58.888481Z</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
@@ -6283,14 +6247,14 @@
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Test TC-090 Passed in 0.14s</t>
+          <t>Test TC-090 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.759440Z</t>
+          <t>2026-06-15T12:49:58.888561Z</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
@@ -6307,7 +6271,7 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.882056Z</t>
+          <t>2026-06-15T12:49:59.049177Z</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
@@ -6317,14 +6281,14 @@
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Test TC-091 Passed in 0.12s</t>
+          <t>Test TC-091 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:49.882134Z</t>
+          <t>2026-06-15T12:49:59.049246Z</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
@@ -6341,7 +6305,7 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.017124Z</t>
+          <t>2026-06-15T12:49:59.229374Z</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
@@ -6351,14 +6315,14 @@
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>Test TC-092 Passed in 0.13s</t>
+          <t>Test TC-092 Passed in 0.18s</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.017184Z</t>
+          <t>2026-06-15T12:49:59.229448Z</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
@@ -6375,7 +6339,7 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.146034Z</t>
+          <t>2026-06-15T12:49:59.392422Z</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
@@ -6385,14 +6349,14 @@
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>Test TC-093 Passed in 0.13s</t>
+          <t>Test TC-093 Passed in 0.16s</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.146122Z</t>
+          <t>2026-06-15T12:49:59.392489Z</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
@@ -6409,7 +6373,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.287095Z</t>
+          <t>2026-06-15T12:49:59.542258Z</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -6419,14 +6383,14 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>Test TC-094 Passed in 0.14s</t>
+          <t>Test TC-094 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.287199Z</t>
+          <t>2026-06-15T12:49:59.542314Z</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -6443,7 +6407,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.407753Z</t>
+          <t>2026-06-15T12:49:59.719132Z</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -6453,14 +6417,14 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>Test TC-095 Passed in 0.12s</t>
+          <t>Test TC-095 Passed in 0.18s</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.407815Z</t>
+          <t>2026-06-15T12:49:59.719205Z</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -6477,7 +6441,7 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.533657Z</t>
+          <t>2026-06-15T12:49:59.900009Z</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
@@ -6487,14 +6451,14 @@
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>Test TC-096 Passed in 0.13s</t>
+          <t>Test TC-096 Passed in 0.18s</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.533713Z</t>
+          <t>2026-06-15T12:49:59.900085Z</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
@@ -6511,7 +6475,7 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.671909Z</t>
+          <t>2026-06-15T12:50:00.075524Z</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
@@ -6521,14 +6485,14 @@
       </c>
       <c r="C195" t="inlineStr">
         <is>
-          <t>Test TC-097 Passed in 0.14s</t>
+          <t>Test TC-097 Passed in 0.18s</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.671965Z</t>
+          <t>2026-06-15T12:50:00.075595Z</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
@@ -6545,7 +6509,7 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.808153Z</t>
+          <t>2026-06-15T12:50:00.224525Z</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
@@ -6555,14 +6519,14 @@
       </c>
       <c r="C197" t="inlineStr">
         <is>
-          <t>Test TC-098 Passed in 0.14s</t>
+          <t>Test TC-098 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.808212Z</t>
+          <t>2026-06-15T12:50:00.224590Z</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -6579,7 +6543,7 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.941679Z</t>
+          <t>2026-06-15T12:50:00.362225Z</t>
         </is>
       </c>
       <c r="B199" t="inlineStr">
@@ -6589,14 +6553,14 @@
       </c>
       <c r="C199" t="inlineStr">
         <is>
-          <t>Test TC-099 Passed in 0.13s</t>
+          <t>Test TC-099 Passed in 0.14s</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:50.941736Z</t>
+          <t>2026-06-15T12:50:00.362289Z</t>
         </is>
       </c>
       <c r="B200" t="inlineStr">
@@ -6613,7 +6577,7 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.079678Z</t>
+          <t>2026-06-15T12:50:00.502650Z</t>
         </is>
       </c>
       <c r="B201" t="inlineStr">
@@ -6630,7 +6594,7 @@
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.079749Z</t>
+          <t>2026-06-15T12:50:00.502712Z</t>
         </is>
       </c>
       <c r="B202" t="inlineStr">
@@ -6647,7 +6611,7 @@
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.225746Z</t>
+          <t>2026-06-15T12:50:00.650957Z</t>
         </is>
       </c>
       <c r="B203" t="inlineStr">
@@ -6664,7 +6628,7 @@
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.225803Z</t>
+          <t>2026-06-15T12:50:00.651044Z</t>
         </is>
       </c>
       <c r="B204" t="inlineStr">
@@ -6681,7 +6645,7 @@
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.354267Z</t>
+          <t>2026-06-15T12:50:00.785348Z</t>
         </is>
       </c>
       <c r="B205" t="inlineStr">
@@ -6698,7 +6662,7 @@
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.354324Z</t>
+          <t>2026-06-15T12:50:00.785430Z</t>
         </is>
       </c>
       <c r="B206" t="inlineStr">
@@ -6715,7 +6679,7 @@
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.474190Z</t>
+          <t>2026-06-15T12:50:00.936648Z</t>
         </is>
       </c>
       <c r="B207" t="inlineStr">
@@ -6725,14 +6689,14 @@
       </c>
       <c r="C207" t="inlineStr">
         <is>
-          <t>Test TC-103 Passed in 0.12s</t>
+          <t>Test TC-103 Passed in 0.15s</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.474247Z</t>
+          <t>2026-06-15T12:50:00.936991Z</t>
         </is>
       </c>
       <c r="B208" t="inlineStr">
@@ -6749,7 +6713,7 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.598539Z</t>
+          <t>2026-06-15T12:50:01.880554Z</t>
         </is>
       </c>
       <c r="B209" t="inlineStr">
@@ -6759,14 +6723,14 @@
       </c>
       <c r="C209" t="inlineStr">
         <is>
-          <t>Test TC-104 Passed in 0.12s</t>
+          <t>Test TC-104 Passed in 0.94s</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>2026-06-15T04:48:51.598606Z</t>
+          <t>2026-06-15T12:50:01.880763Z</t>
         </is>
       </c>
       <c r="B210" t="inlineStr">
@@ -6885,7 +6849,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Failed</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="E4" t="inlineStr"/>

</xml_diff>